<commit_message>
Simplify Luca model to case-brief assumptions only; update board deck and tracker to match
Co-authored-by: JoaoTavarees <JoaoTavarees@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/luca_chief_of_staff_case/deliverables/Luca_Content_Pipeline_Master_Tracker.xlsx
+++ b/luca_chief_of_staff_case/deliverables/Luca_Content_Pipeline_Master_Tracker.xlsx
@@ -1299,7 +1299,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Rafa (Synthesia)</t>
+          <t>Synthesia Specialist 1</t>
         </is>
       </c>
       <c r="G10" s="11" t="n">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>Elena (Sound)</t>
+          <t>Sound Editor 1</t>
         </is>
       </c>
       <c r="G11" s="11" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Rafa (Synthesia)</t>
+          <t>Synthesia Specialist 1</t>
         </is>
       </c>
       <c r="G12" s="11" t="n">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Valeria (Motion)</t>
+          <t>Motion Designer 2</t>
         </is>
       </c>
       <c r="G13" s="11" t="n">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>Valeria (Motion)</t>
+          <t>Motion Designer 2</t>
         </is>
       </c>
       <c r="G14" s="11" t="n">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Valeria (Motion)</t>
+          <t>Motion Designer 2</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Jorge (Motion)</t>
+          <t>Motion Designer 1</t>
         </is>
       </c>
       <c r="G16" s="11" t="n">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>Valeria (Motion)</t>
+          <t>Motion Designer 2</t>
         </is>
       </c>
       <c r="G17" s="11" t="n">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Valeria (Motion)</t>
+          <t>Motion Designer 2</t>
         </is>
       </c>
       <c r="G18" s="11" t="n">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Jorge (Motion)</t>
+          <t>Motion Designer 1</t>
         </is>
       </c>
       <c r="G19" s="11" t="n">
@@ -2419,7 +2419,7 @@
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>Pablo (Design)</t>
+          <t>Graphic Designer 2</t>
         </is>
       </c>
       <c r="G20" s="11" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>Carla (Design)</t>
+          <t>Graphic Designer 1</t>
         </is>
       </c>
       <c r="G21" s="11" t="n">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>Carla (Design)</t>
+          <t>Graphic Designer 1</t>
         </is>
       </c>
       <c r="G22" s="11" t="n">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
-          <t>Pablo (Design)</t>
+          <t>Graphic Designer 2</t>
         </is>
       </c>
       <c r="G23" s="11" t="n">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>Pablo (Design)</t>
+          <t>Graphic Designer 2</t>
         </is>
       </c>
       <c r="G24" s="11" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>Diego (Script)</t>
+          <t>Scriptwriter 2</t>
         </is>
       </c>
       <c r="G25" s="11" t="n">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>Sofía (Script)</t>
+          <t>Scriptwriter 1</t>
         </is>
       </c>
       <c r="G26" s="11" t="n">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>Mariana (Script)</t>
+          <t>Scriptwriter 3</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>Diego (Script)</t>
+          <t>Scriptwriter 2</t>
         </is>
       </c>
       <c r="G28" s="11" t="n">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>Diego (Script)</t>
+          <t>Scriptwriter 2</t>
         </is>
       </c>
       <c r="G29" s="11" t="n">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>Sofía (Script)</t>
+          <t>Scriptwriter 1</t>
         </is>
       </c>
       <c r="G30" s="11" t="n">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>Sofía (Script)</t>
+          <t>Scriptwriter 1</t>
         </is>
       </c>
       <c r="G31" s="11" t="n">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t>Sofía (Script)</t>
+          <t>Scriptwriter 1</t>
         </is>
       </c>
       <c r="G32" s="11" t="n">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>Sofía (Script)</t>
+          <t>Scriptwriter 1</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
@@ -3357,7 +3357,7 @@
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
-          <t>Mariana (Script)</t>
+          <t>Scriptwriter 3</t>
         </is>
       </c>
       <c r="G34" s="11" t="n">
@@ -3424,7 +3424,7 @@
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>Diego (Script)</t>
+          <t>Scriptwriter 2</t>
         </is>
       </c>
       <c r="G35" s="11" t="n">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t>Sofía (Script)</t>
+          <t>Scriptwriter 1</t>
         </is>
       </c>
       <c r="G36" s="11" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t>Mariana (Script)</t>
+          <t>Scriptwriter 3</t>
         </is>
       </c>
       <c r="G37" s="11" t="n">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="F38" s="10" t="inlineStr">
         <is>
-          <t>Mariana (Script)</t>
+          <t>Scriptwriter 3</t>
         </is>
       </c>
       <c r="G38" s="11" t="n">
@@ -3692,7 +3692,7 @@
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>Sofía (Script)</t>
+          <t>Scriptwriter 1</t>
         </is>
       </c>
       <c r="G39" s="11" t="n">

</xml_diff>